<commit_message>
docs: document hotel agent architecture setup and demo workflow
</commit_message>
<xml_diff>
--- a/data/hotel_prices.xlsx
+++ b/data/hotel_prices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1572,6 +1572,117 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>全季成都高新电子科大酒店</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6117313</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>舒压-高级大床房</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>￥489</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:45:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>全季成都高新电子科大酒店</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>6117313</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>豪华大床房</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>￥529</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:45:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>全季成都高新电子科大酒店</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>6117313</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>大床房</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>￥429</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:45:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>